<commit_message>
Update leads tracker 2026-09-09
</commit_message>
<xml_diff>
--- a/leads_tracker.xlsx
+++ b/leads_tracker.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -632,11 +632,6 @@
           <t>Fraser River Tunnel Project (George Massey Replacement) — Re-Tender for Major Construction</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
           <t>Surrey Now-Leader / BC Ministry of Transportation and Infrastructure</t>
@@ -679,11 +674,6 @@
           <t>Yellowhead Copper Mine (Trekor Metals) — Infrastructure &amp; Civil Engineering Work Package</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>Mining Weekly / BC Gov News / Trekor Metals</t>
@@ -726,11 +716,6 @@
           <t>Canagold New Polaris Gold-Antimony Mine — Construction &amp; Engineering Services</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>Newsfile Corp / BC Gov News (Look West update)</t>
@@ -773,11 +758,6 @@
           <t>BC Hydro Grid-Scale Battery Energy Storage System (BESS) — Request for Supplier Qualifications</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>BC Hydro / T-Net News</t>
@@ -820,11 +800,6 @@
           <t>Metro Vancouver Iona Island Wastewater Treatment Plant — Standby Power System Facility</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
           <t>Metro Vancouver Bids &amp; Tenders / TendersOnTime</t>
@@ -867,11 +842,6 @@
           <t>Federal Airports Capital Assistance Program — Six BC Airport Infrastructure Projects ($23.5M)</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
           <t>Transport Canada / Canada.ca</t>
@@ -895,6 +865,288 @@
       <c r="M9" t="inlineStr">
         <is>
           <t>Transport Canada announced August 26, 2026 that over $23.5 million will fund critical infrastructure improvements at six BC airports through the Airports Capital Assistance Program; individual airport authorities will now procure civil and structural construction services locally.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Fraser River Tunnel Project – Remaining Three Construction Work Packages</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>BC Gov News / Infrastructure BC</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>https://news.gov.bc.ca/releases/2026TT0066-000796</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Register on Infrastructure BC's project mailing list at infrastructurebc.com/project/fraser-river-tunnel-project, monitor BC Bid for RFQ/RFP postings, and pre-position your prequalification package now targeting the tunnel elements, marine works, and highway connector packages slated for 2027 procurement.</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>BC's $8.5B immersed-tube tunnel replacing the George Massey Tunnel will procure three additional multi-hundred-million-dollar civil/structural work packages in 2027, following the first two RFPs issued in August 2026; EAO review expected to conclude before end of 2026 unlocking major construction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Iona Island Wastewater Treatment Plant – Phase 2 Major Construction Packages</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Metro Vancouver / ReNew Canada</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>https://metrovancouver.org/services/liquid-waste/iona-island-wastewater-treatment-plant-projects</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Register on Metro Vancouver's Iona Projects mailing list at metrovancouver.org, set up commodity-code alerts on metrovancouver.bidsandtenders.ca for civil/structural/mechanical works, and engage Metro Vancouver's Purchasing Admin (purchasing_admin@metrovancouver.org) to express interest in upcoming design-build and CM-at-Risk packages.</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Metro Vancouver's $6B upgrade of the Iona Island WWTP (serving 875,000+ residents) is in early works and preliminary design; Phase 2 treatment plant and related civil/structural works packages are expected to begin procurement in 2026–2027, with construction ramping up through 2034.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Canagold New Polaris Gold-Antimony Mine – BC EAO Under Review, Construction Decision ~2028</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Canagold Resources / BC EAO Project Registry</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>https://www.newsfilecorp.com/release/290842/Canagold-Submits-Environmental-Application-for-the-New-Polaris-Project</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Monitor the BC EAO project registry for the New Polaris application milestones; contact Canagold's President &amp; COO Garry Biles, P.Eng. to introduce civil/mining construction capabilities and express interest in early contractor engagement for access road, camp, and underground development packages.</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Canagold (TSX: CCM) filed an EA application with the BC EAO on April 1, 2026 for its $757M New Polaris underground gold-antimony mine in northern BC; feasibility complete with 47% IRR; BC priority-project status granted May 2026; construction targeted for 2028 requiring roads, camp, portal, and mill infrastructure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>MoTT Project 38447-0000 – Highway 97 Coulee Creek Culvert Replacement</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>BC Ministry of Transportation and Transit – Unofficial Tender Documents / BC Bid</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>https://www2.gov.bc.ca/gov/content/transportation/transportation-infrastructure/contracting-to-transportation/highway-bridge-construction/unofficial-tender-documents</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Download the tender package immediately from BC Bid (search Project No. 38447-0000), confirm closing date with the ministry contact listed in the solicitation, and mobilize estimating resources for a fall 2026 construction window.</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>BC Ministry of Transportation and Transit (MoTT) has posted an Invitation to Tender for culvert replacement on Highway 97 at Coulee Creek; listed on the MoTT Unofficial Tender Documents page and available for download via BC Bid, targeting a 2026/27 construction season.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>MoTT Project 38610-0000 – Asphalt Surfacing 2026/27 Hwy 16 Kasiks River to Andesite Boat Launch (41.1 Lane Km)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>BC Ministry of Transportation and Transit – Unofficial Tender Documents / BC Bid</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>https://www2.gov.bc.ca/gov/content/transportation/transportation-infrastructure/contracting-to-transportation/highway-bridge-construction/unofficial-tender-documents</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Download tender documents from BC Bid (Project No. 38610-0000), verify closing date with the district contact in the solicitation, and line up asphalt plant and paving crew availability for a late-season mobilization in the Skeena District.</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>BC MoTT Invitation to Tender for asphalt surfacing along a 41.1-lane-km stretch of Highway 16 in northwestern BC for the 2026/27 season; posted on the MoTT Unofficial Tender Documents page and open on BC Bid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>North Coast Transmission Line Phase 1 – Ongoing Subcontractor &amp; Supply Opportunities (BC Hydro / BC Bid)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>BC Hydro / Journal of Commerce</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>https://www.bchydro.com/energy-in-bc/projects/north-coast-bc-electrification/construction.html</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Register or confirm your standing on BC Hydro's Civil Contractor Registry (bchydro.com/work-with-us/suppliers), email NCTLproject@bchydro.com to flag interest in civil works packages, and monitor BC Bid for related RFPs covering access roads, camp construction, and equipment services along the Prince George–Fraser Lake corridor.</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>BC Hydro's $6B North Coast Transmission Line (Prince George to Terrace, 165 km of new 500 kV line) broke ground in July 2026; BC Hydro is actively sourcing civil contractors, camp services, road builders, and supply through BC Bid and its civil contractor registry as construction ramps through Q4 2026.</t>
         </is>
       </c>
     </row>
@@ -909,7 +1161,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1070,13 +1322,11 @@
           <t>Stuart McDonald</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>Trekor Metals Limited (TSX: TKO)</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>Trekor Metals / GlobeNewswire</t>
@@ -1087,8 +1337,6 @@
           <t>https://finance.yahoo.com/economy/articles/trekor-advances-environmental-assessment-yellowhead-123000463.html</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -1116,13 +1364,11 @@
           <t>Catalin Kilofliski</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>Canagold Resources Ltd. (TSX: CCM)</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>Newsfile Corp / Canagold Resources</t>
@@ -1133,8 +1379,6 @@
           <t>https://www.newsfilecorp.com/release/295407/Canagold-New-Polaris-GoldAntimony-Project-Recognized-as-a-Priority-Project-by-British-Columbia</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -1162,13 +1406,11 @@
           <t>Mark Liedemann</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>Infrastructure BC</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>ReNew Canada / Infrastructure BC</t>
@@ -1179,8 +1421,6 @@
           <t>https://www.renewcanada.net/latest-edition-of-bc-major-infrastructure-projects-brochure-released/</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -1194,6 +1434,144 @@
       <c r="L6" t="inlineStr">
         <is>
           <t>Liedemann oversees BC's major public infrastructure procurement pipeline — including the Iona Island WWTP ($6B), Surrey-Langley SkyTrain ($6B), Fraser River Tunnel ($4.15B), and the Cowichan and Dawson Creek hospital redevelopments — and publishes the BC Major Infrastructure Projects Brochure that is the authoritative forward view for contractors; he is the gateway relationship for the province's $37.7B three-year capital program.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Brian G. Thurston, P.Geo.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Copper Quest Exploration Inc. (CSE: CQX)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Copper Quest / IRW Press</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>https://irw-press.com/en/copper-quest-receives-kitimat-copper-gold-project-exploration-permit</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Email Copper Quest's corporate office in Vancouver this week referencing the September 9 exploration permit announcement; offer a brief capability deck covering BC drill-access road construction, remote camp setup, and geophysical line-cutting crews to position ahead of their fall 2026 field program.</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Thurston is the technical decision-maker and qualified person behind the newly permitted Kitimat Copper-Gold Project in northwestern BC. With drilling and geophysics set to begin in September 2026, he is the direct contact for exploration services, access roads, camp logistics, and drill-contractor engagement on a freshly permitted 6,800-hectare Skeena Division porphyry target.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Catalin Kilofliski</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Canagold Resources Ltd. (TSX: CCM)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Canagold Resources / Newsfile Corp</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>https://canagoldresources.com/</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Reach out via Canagold's Vancouver investor relations contact referencing the April 2026 EA filing and BC priority status; propose an introductory call to discuss early civil engineering support for access road assessment, marine landing studies, and camp infrastructure scoping as the EAO review advances.</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Kilofliski is leading the BC EAO review of the $757M New Polaris gold-antimony mine in northern BC, which achieved BC priority-project status in May 2026 and targets a 2028 construction decision. He is the strategic contact for pre-FEED civil, geotechnical, and access-road engineering mandates ahead of formal contractor procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Mark Liedemann</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Infrastructure BC</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Infrastructure BC / ReNew Canada</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>https://www.infrastructurebc.com/publications/bc-infrastructure-project-brochure/</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Request the 2026 Spring BC Major Infrastructure Projects Brochure from infrastructurebc.com and attend Infrastructure BC's next industry engagement session; send a brief firm profile to Infrastructure BC's communications team citing interest in the Fraser River Tunnel remaining packages and Iona WWTP Phase 2 civil works, referencing the multi-package procurement model now in use.</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Liedemann leads Infrastructure BC, the provincial centre of expertise that oversees procurement for BC's major public infrastructure projects including the Fraser River Tunnel (remaining 3 of 5 packages), Iona Island WWTP Phase 2, and the $52B provincial infrastructure pipeline featured in the 2026 Spring BC Major Infrastructure Projects Brochure. He is the highest-leverage relationship for BC's major civil and structural pipeline.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update leads tracker 2026-09-16
</commit_message>
<xml_diff>
--- a/leads_tracker.xlsx
+++ b/leads_tracker.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -884,11 +884,6 @@
           <t>Fraser River Tunnel Project – Remaining Three Construction Work Packages</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
           <t>BC Gov News / Infrastructure BC</t>
@@ -931,11 +926,6 @@
           <t>Iona Island Wastewater Treatment Plant – Phase 2 Major Construction Packages</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
           <t>Metro Vancouver / ReNew Canada</t>
@@ -978,11 +968,6 @@
           <t>Canagold New Polaris Gold-Antimony Mine – BC EAO Under Review, Construction Decision ~2028</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
           <t>Canagold Resources / BC EAO Project Registry</t>
@@ -1025,11 +1010,6 @@
           <t>MoTT Project 38447-0000 – Highway 97 Coulee Creek Culvert Replacement</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
           <t>BC Ministry of Transportation and Transit – Unofficial Tender Documents / BC Bid</t>
@@ -1072,11 +1052,6 @@
           <t>MoTT Project 38610-0000 – Asphalt Surfacing 2026/27 Hwy 16 Kasiks River to Andesite Boat Launch (41.1 Lane Km)</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
           <t>BC Ministry of Transportation and Transit – Unofficial Tender Documents / BC Bid</t>
@@ -1119,11 +1094,6 @@
           <t>North Coast Transmission Line Phase 1 – Ongoing Subcontractor &amp; Supply Opportunities (BC Hydro / BC Bid)</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>BC Hydro / Journal of Commerce</t>
@@ -1147,6 +1117,288 @@
       <c r="M15" t="inlineStr">
         <is>
           <t>BC Hydro's $6B North Coast Transmission Line (Prince George to Terrace, 165 km of new 500 kV line) broke ground in July 2026; BC Hydro is actively sourcing civil contractors, camp services, road builders, and supply through BC Bid and its civil contractor registry as construction ramps through Q4 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Newmont Red Chris Block Cave Underground Mine — Construction Packages</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>BC Gov News / Mining News North</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>https://news.gov.bc.ca/releases/2026MCM0029-000727</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Contact Newmont's Vancouver investor-relations office (investor.relations@newmont.com / 604-558-1784) and JV partner Imperial Metals to pre-position as a civil, underground development, or site-services contractor ahead of anticipated FID and early works RFQ release Q4 2026.</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Newmont received key BC regulatory approvals in June 2026 for the Red Chris open-pit-to-block-cave transition; a Final Investment Decision is expected in late 2026, which would trigger over $1.8B in underground civil and mining construction in BC's Golden Triangle with 1,800+ construction jobs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>BC Hydro North Coast Transmission Line (NCTL) — Phase 2 Construction Procurement</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>BC Hydro / BC Gov News</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>https://www.bchydro.com/energy-in-bc/projects/north-coast-bc-electrification/jobs-opportunities.html</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Register on BC Bid and monitor NCTLproject@bchydro.com for Phase 2 RFQ/RFP notices; contact the BC Hydro NCTL project office at 1-866-647-3334 to get on the contractor engagement list before Phase 2 procurement opens.</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Phase 1 construction (Prince George to Glenannan) broke ground September 2026 under a $3.9B federal-provincial commitment; Phase 2 toward Terrace is expected to begin procurement in 2027, requiring heavy civil, access-road, and tower-erection contractors across northern BC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Iona Island Wastewater Treatment Plant — Phase 2 Major Works Procurement (~$6B)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Metro Vancouver / ReNew Canada</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>https://metrovancouver.org/services/liquid-waste/iona-island-wastewater-treatment-plant-projects</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Request a copy of Metro Vancouver's project definition documents and engage AECOM (Engineer of Record) and the Metro Vancouver Procurement team early to understand work-packaging strategy and prequalification requirements.</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Metro Vancouver's Board endorsed a revised $6B phased upgrade in Oct 2025; Phase 1 early works and foundations are wrapping up in 2026, and the bulk of main treatment-plant construction packages covering secondary-treatment civils are anticipated to go to tender in 2027–2028.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Surrey Langley SkyTrain — Ongoing Civil/Guideway &amp; Station Construction Sub-Trade Work</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>BC Gov News / AtkinsRéalis / BC Bid</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>https://surreylangleyskytrain.gov.bc.ca/news-releases/</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Contact SkyLink Guideway Partners (Dragados/Ledcor JV) and South Fraser Station Partners directly for active sub-trade RFQs; also monitor BC Bid for utility-relocation and civil ancillary packages issued by the Province.</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>All three prime contracts for the $6B+ Surrey Langley SkyTrain (guideway, stations, systems/trackwork) are awarded and active; SkyLink Guideway Partners and South Fraser Station Partners are actively tendering sub-trade and civil packages as construction peaks in 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>North Shore Wastewater Treatment Plant — Mechanical/Electrical Sub-Trade Work Packages</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Richmond News / ES&amp;E Magazine</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>https://www.richmond-news.com/highlights/photos-metro-vancouver-offers-look-inside-north-shore-sewage-plant-as-new-contractor-confirmed-10153164</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Contact PCL Constructors Westcoast VP Travis Chorney and their procurement team directly in North Vancouver to request inclusion on the sub-trade bid list; AECOM is Engineer of Record for design-coordination queries.</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>PCL Constructors Westcoast is the GC on the $3.86B North Shore WWTP; site activity is peaking through 2026–2027 with 650+ tradespeople needed to install 40,000 m of pipe and 800 km of electrical on the North Vancouver site, with ongoing sub-trade package releases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Record Ridge Industrial Mineral Mine — Site Preparation &amp; Civil Construction, near Rossland BC</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>West High Yield Resources / StockTitan</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>https://www.stocktitan.net/news/WHYRF/west-high-yield-resources-receives-occupant-licence-to-cut-and-mt0rf3i70nl3.html</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Contact Frank Marasco, President and CEO of West High Yield Resources, and primary contractor Skemxist Solutions regarding early civil, access-road, and site-prep packages; move quickly as the company has indicated imminent construction mobilization.</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>West High Yield Resources received its Occupant Licence to Cut timber (50 ha) on September 16, 2026, following its BC Mines Act and highway access permits; the company is now advancing toward timber clearing, access-road construction, and site earthworks with commercial production targeted for 2029.</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1448,13 +1700,11 @@
           <t>Brian G. Thurston, P.Geo.</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>Copper Quest Exploration Inc. (CSE: CQX)</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>Copper Quest / IRW Press</t>
@@ -1465,8 +1715,6 @@
           <t>https://irw-press.com/en/copper-quest-receives-kitimat-copper-gold-project-exploration-permit</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -1494,13 +1742,11 @@
           <t>Catalin Kilofliski</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
           <t>Canagold Resources Ltd. (TSX: CCM)</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>Canagold Resources / Newsfile Corp</t>
@@ -1511,8 +1757,6 @@
           <t>https://canagoldresources.com/</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -1540,13 +1784,11 @@
           <t>Mark Liedemann</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>Infrastructure BC</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>Infrastructure BC / ReNew Canada</t>
@@ -1557,8 +1799,6 @@
           <t>https://www.infrastructurebc.com/publications/bc-infrastructure-project-brochure/</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -1572,6 +1812,144 @@
       <c r="L9" t="inlineStr">
         <is>
           <t>Liedemann leads Infrastructure BC, the provincial centre of expertise that oversees procurement for BC's major public infrastructure projects including the Fraser River Tunnel (remaining 3 of 5 packages), Iona Island WWTP Phase 2, and the $52B provincial infrastructure pipeline featured in the 2026 Spring BC Major Infrastructure Projects Brochure. He is the highest-leverage relationship for BC's major civil and structural pipeline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>David Thornton</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Newmont Corporation (Red Chris Mine, Golden Triangle BC)</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Business in Vancouver</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>https://www.biv.com/news/bc-mining-racking-up-wins-as-new-mines-expansions-move-ahead-11804192</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Reach out via Newmont's Vancouver office (604-558-1784) with a targeted capability statement covering underground civil works, concrete, and surface infrastructure; reference the FID timeline and offer to present at Newmont's contractor pre-qualification sessions.</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>As Newmont's Managing Director for Red Chris, Thornton is the executive steering the block cave FID process and will be central to early-works and construction contractor engagement. With a FID expected in H2 2026 and 1,800 construction jobs on the line, he is the key gatekeeper for civil and underground mining contract awards.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Frank Marasco</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>West High Yield Resources Ltd. (TSXV: WHY)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>West High Yield Resources / InvestorNews</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>https://whyresources.com/record-ridge-magnesium-project/</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Contact Marasco directly through West High Yield's Calgary corporate office with a site-preparation and access-road construction capability brief; also reach out to primary contractor Skemxist Solutions, who is managing procurement and commissioning, to position for sub-trade work.</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Marasco is leading Record Ridge toward imminent construction mobilization following three major BC permits secured in 2025–2026. Detailed engineering is underway with firms Fuse, SRK, and McElhanney; Marasco controls the contractor and civil construction decisions for this BC critical minerals project.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Mark Liedemann</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Infrastructure BC</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>ReNew Canada / Infrastructure BC</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>https://www.infrastructurebc.com/publications/bc-infrastructure-project-brochure/</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Request a copy of the 2026 Spring BC Major Infrastructure Projects Brochure from Infrastructure BC and seek a firm introduction meeting with Liedemann's team; register for Infrastructure BC's procurement outreach events to get early sight lines on upcoming RFQs for the Iona Island, health capital, and transit pipeline.</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Liedemann oversees BC's major infrastructure procurement pipeline across all $52B+ of provincially-significant projects, including transit, health, and energy. He released the 2026 Spring BC Major Infrastructure Projects Brochure in May and is the central figure coordinating collaborative contracting across all P3 and Design-Build procurement in BC.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update leads tracker 2026-09-30
</commit_message>
<xml_diff>
--- a/leads_tracker.xlsx
+++ b/leads_tracker.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:M27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1136,11 +1136,6 @@
           <t>Newmont Red Chris Block Cave Underground Mine — Construction Packages</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>BC Gov News / Mining News North</t>
@@ -1183,11 +1178,6 @@
           <t>BC Hydro North Coast Transmission Line (NCTL) — Phase 2 Construction Procurement</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
           <t>BC Hydro / BC Gov News</t>
@@ -1230,11 +1220,6 @@
           <t>Iona Island Wastewater Treatment Plant — Phase 2 Major Works Procurement (~$6B)</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
           <t>Metro Vancouver / ReNew Canada</t>
@@ -1277,11 +1262,6 @@
           <t>Surrey Langley SkyTrain — Ongoing Civil/Guideway &amp; Station Construction Sub-Trade Work</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>BC Gov News / AtkinsRéalis / BC Bid</t>
@@ -1324,11 +1304,6 @@
           <t>North Shore Wastewater Treatment Plant — Mechanical/Electrical Sub-Trade Work Packages</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
           <t>Richmond News / ES&amp;E Magazine</t>
@@ -1371,11 +1346,6 @@
           <t>Record Ridge Industrial Mineral Mine — Site Preparation &amp; Civil Construction, near Rossland BC</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>West High Yield Resources / StockTitan</t>
@@ -1399,6 +1369,288 @@
       <c r="M21" t="inlineStr">
         <is>
           <t>West High Yield Resources received its Occupant Licence to Cut timber (50 ha) on September 16, 2026, following its BC Mines Act and highway access permits; the company is now advancing toward timber clearing, access-road construction, and site earthworks with commercial production targeted for 2029.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>BC Hydro West End Underground Substation — Vancouver (~$1B Heavy Civil &amp; Electrical)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Journal of Commerce / BC Gov News</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>https://canada.constructconnect.com/joc/news/infrastructure/2026/09/new-substations-slated-for-downtown-vancouver-one-will-be-built-underground</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Monitor BCUC proceeding (Application ID 1396) for certificate decision expected October 30, 2026; pre-position with BC Hydro's civil procurement team and review WSP/Kasian design documents to prepare a pre-qualification package for deep excavation and underground structural scope.</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>BC Hydro is seeking BCUC approval for a $1.028B underground substation at 1150 Nelson Street in Vancouver's West End, targeting a construction start in late 2026 pending a regulatory decision expected by October 30, 2026; this is a massive excavation, structural concrete, and electrical infrastructure project.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Surge Copper Berg Project — Central BC ($4.7B Copper-Moly Mine, Early EA Stage)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>GlobeNewswire / BC EAO</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>https://www.globenewswire.com/news-release/2026/09/16/3363033/0/en/surge-copper-commences-environmental-assessment-process-for-berg-copper-project.html</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Engage Surge Copper CEO Leif Nilsson and technical teams now during the Early Engagement phase; offer geotechnical drilling, infrastructure planning, or environmental baseline support — relationships established at this stage typically carry through to construction contracting.</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Surge Copper's Initial Project Description for the $4.7B Berg copper-molybdenum-silver-gold project in central BC was accepted by the BC EAO and the Impact Assessment Agency of Canada on September 9, 2026, commencing the Early Engagement phase; the project includes a 120,000 t/d concentrator and a new 230 kV transmission line — major civil, structural, and mining infrastructure tendering is 3–6 years out but early consultant relationships matter now.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Iona Island WWTP Secondary Upgrade — Metro Vancouver (~$6B Heavy Civil, Tendering from ~2027)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>ReNew Canada / Metro Vancouver Bids &amp; Tenders</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>https://www.renewcanada.net/metro-vancouver-adopts-new-approach-for-upgrading-the-iona-island-wwtp/</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Register on Metro Vancouver's bids and tenders portal (metrovancouver.bidsandtenders.ca) and monitor for Phase 1 civil works sub-packages; reach out to Jacobs and AECOM local offices to position as a sub-consultant or civil sub-trade for the foundation and site preparation scope.</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Metro Vancouver's redesigned $6B secondary treatment upgrade at Iona Island (Richmond) is in preliminary design with Jacobs/AECOM JV; Phase 1 ($750M in site preparation, ground foundations, and civil works on soft Fraser River delta soils) is fully funded and construction packages are expected to go to market progressively from 2027.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>MERX — Devonshire Catchment Sanitary Sewer Upgrades, Township of Esquimalt (ENG 26-05)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>MERX</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>https://www.merx.com/public/solicitations/british-columbia-379</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Download RFP documents from MERX (solicitation 444174286497), assemble a civil/environmental engineering team familiar with Esquimalt's existing sewer infrastructure, and submit before the October 28, 2026 deadline.</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Township of Esquimalt is seeking consulting engineering services for the Devonshire Catchment Sanitary Sewer Upgrades — a civil/underground sewer infrastructure project on southern Vancouver Island; published September 25, 2026, closing October 28, 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>City of Vancouver — Strathcona HDD &amp; Underground Electrical Upgrades Ph 2 &amp; 2A (ITT PS20261865-ENG-ITT)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>City of Vancouver Procurement</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>https://bids.sciquest.com/apps/Router/PublicEvent?CustomerOrg=CityofVancouver</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Obtain ITT documents from the City of Vancouver procurement portal (contact Amjid Qazi at Amjid.Qazi@vancouver.ca), confirm HDD equipment availability, and submit before October 9, 2026 at 3:00 PM PDT.</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>City of Vancouver is inviting qualified contractors to deliver trenchless HDD construction, HDPE conduit installation, and surface restoration for the Strathcona underground electrical upgrade Phases 2 and 2A — heavy civil/trenchless scope; closes October 9, 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>City of White Rock — Consulting Services for Goggs Ave Watermain &amp; Sanitary Sewer (WR26-030)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>MERX</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>https://www.merx.com/public/solicitations/british-columbia-379</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Download RFP documents from MERX (solicitation 444174163175), prepare a team with water and sanitary sewer design experience in Metro Vancouver's South of Fraser municipalities, and respond before the November 2, 2026 closing date.</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>City of White Rock is seeking a civil engineering consultant for watermain and sanitary sewer design along Goggs Avenue from Maple to Kent — a civil/structural underground infrastructure project; published September 25, 2026, closing November 2, 2026.</t>
         </is>
       </c>
     </row>
@@ -1413,7 +1665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1826,13 +2078,11 @@
           <t>David Thornton</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
           <t>Newmont Corporation (Red Chris Mine, Golden Triangle BC)</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>Business in Vancouver</t>
@@ -1843,8 +2093,6 @@
           <t>https://www.biv.com/news/bc-mining-racking-up-wins-as-new-mines-expansions-move-ahead-11804192</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -1872,13 +2120,11 @@
           <t>Frank Marasco</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>West High Yield Resources Ltd. (TSXV: WHY)</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>West High Yield Resources / InvestorNews</t>
@@ -1889,8 +2135,6 @@
           <t>https://whyresources.com/record-ridge-magnesium-project/</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -1918,13 +2162,11 @@
           <t>Mark Liedemann</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>Infrastructure BC</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>ReNew Canada / Infrastructure BC</t>
@@ -1935,8 +2177,6 @@
           <t>https://www.infrastructurebc.com/publications/bc-infrastructure-project-brochure/</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -1950,6 +2190,144 @@
       <c r="L12" t="inlineStr">
         <is>
           <t>Liedemann oversees BC's major infrastructure procurement pipeline across all $52B+ of provincially-significant projects, including transit, health, and energy. He released the 2026 Spring BC Major Infrastructure Projects Brochure in May and is the central figure coordinating collaborative contracting across all P3 and Design-Build procurement in BC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>JDS Energy &amp; Mining — Project Delivery Leadership</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>JDS Energy &amp; Mining Inc.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>GlobeNewswire / International Mining</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>https://im-mining.com/2026/02/10/osisko-development-enlists-jds-for-cariboo-gold-project-build/</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Reach out to JDS Energy &amp; Mining's Vancouver office this week; introduce your firm's underground civil, earthworks, or structural capabilities and request inclusion on their pre-qualified sub-trade list for Cariboo — earthworks, portal construction, water management, and bridge scopes are actively tendering.</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>JDS Energy &amp; Mining holds the Project and Construction Management Services contract for Osisko Gold's $990M Cariboo Gold Project in central BC; their VP of Project Delivery and procurement team are currently awarding civil, structural, and underground infrastructure sub-packages as the project ramps to full construction. JDS is the key gatekeeper for all major civil sub-trade opportunities at Cariboo through 2028.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Leif Nilsson</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Surge Copper Corp.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>GlobeNewswire / Surge Copper</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>https://www.globenewswire.com/news-release/2026/09/16/3363033/0/en/surge-copper-commences-environmental-assessment-process-for-berg-copper-project.html</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Contact Surge Copper's Vancouver office and request a meeting with Leif Nilsson or the Berg Project's engineering lead; position your firm's geotechnical, access road, or civil site assessment capabilities as support for the 2027 feasibility-level engineering and EA field programs — this is the optimal entry window before major contracts are structured.</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Leif Nilsson leads Surge Copper's $4.7B Berg Copper Project in central BC through its newly commenced provincial and federal environmental assessment process — the project entered the EAO Early Engagement phase September 16, 2026. Nilsson is the primary decision-maker for all technical, environmental, and engagement contracting over the next 2–3 years of EA and feasibility work, including geotechnical, infrastructure planning, and civil access studies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Jeanine Martin</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Vancouver Regional Construction Association (VRCA)</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Journal of Commerce / VRCA</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>https://canada.constructconnect.com/joc/news/government/2026/09/b-c-construction-leaders-seek-certainty-amid-election-instability</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Attend upcoming VRCA election advocacy events and member roundtables in October 2026; engage Jeanine Martin directly on prompt payment and procurement reform issues — visibility with VRCA leadership positions your firm favorably with both public clients and the incoming government's infrastructure advisory process.</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Jeanine Martin, as VRCA president, is leading the industry's post-election advocacy campaign for stable infrastructure procurement and prompt payment legislation in BC; she is actively meeting with all provincial party leaders and candidates ahead of the October 24, 2026 election and is a central connector to Metro Vancouver's major public client network, including TransLink, Metro Vancouver, and the BC Ministry of Transportation.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update leads tracker 2026-10-07
</commit_message>
<xml_diff>
--- a/leads_tracker.xlsx
+++ b/leads_tracker.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M27"/>
+  <dimension ref="A1:M33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1388,11 +1388,6 @@
           <t>BC Hydro West End Underground Substation — Vancouver (~$1B Heavy Civil &amp; Electrical)</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
           <t>Journal of Commerce / BC Gov News</t>
@@ -1435,11 +1430,6 @@
           <t>Surge Copper Berg Project — Central BC ($4.7B Copper-Moly Mine, Early EA Stage)</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
           <t>GlobeNewswire / BC EAO</t>
@@ -1482,11 +1472,6 @@
           <t>Iona Island WWTP Secondary Upgrade — Metro Vancouver (~$6B Heavy Civil, Tendering from ~2027)</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
           <t>ReNew Canada / Metro Vancouver Bids &amp; Tenders</t>
@@ -1529,11 +1514,6 @@
           <t>MERX — Devonshire Catchment Sanitary Sewer Upgrades, Township of Esquimalt (ENG 26-05)</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
           <t>MERX</t>
@@ -1576,11 +1556,6 @@
           <t>City of Vancouver — Strathcona HDD &amp; Underground Electrical Upgrades Ph 2 &amp; 2A (ITT PS20261865-ENG-ITT)</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
           <t>City of Vancouver Procurement</t>
@@ -1623,11 +1598,6 @@
           <t>City of White Rock — Consulting Services for Goggs Ave Watermain &amp; Sanitary Sewer (WR26-030)</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
           <t>MERX</t>
@@ -1651,6 +1621,288 @@
       <c r="M27" t="inlineStr">
         <is>
           <t>City of White Rock is seeking a civil engineering consultant for watermain and sanitary sewer design along Goggs Avenue from Maple to Kent — a civil/structural underground infrastructure project; published September 25, 2026, closing November 2, 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Fraser River Tunnel Project – Remaining Three Civil Construction Packages (GC-3 through GC-5)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>BC Gov News / Infrastructure BC / ENR</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>https://news.gov.bc.ca/releases/2026TT0058-000706</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Register on BC Bid and Infrastructure BC's portal immediately; review GC-1/GC-2 RFQ documents to align your pre-qualification package with the scope of the remaining three packages before their 2027 release. Engage Transportation Investment Corporation (TI Corp) as the delivery agency.</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>BC terminated its original progressive design-build contract in June 2026 and re-tendered the $8.5B George Massey Tunnel replacement as five separate packages; the first two RFQs (immersed tube/south portal and north portal) closed August 2026, with RFPs expected by early 2027 and three more packages (tunnel fit-out, Deas Slough Bridge, and highway/civil works) to be procured through 2027.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Iona Island Wastewater Treatment Plant Upgrade – Phase 2 Major Construction Packages (Metro Vancouver)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Metro Vancouver / Water Canada / ReNew Canada</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>https://www.renewcanada.net/the-projects/iona-island-wastewater-treatment-plant/</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Monitor Metro Vancouver's bids&amp;tenders portal (metrovancouver.bidsandtenders.ca) weekly for new ITT/RFQ postings; contact Metro Vancouver Procurement Division to pre-qualify for civil/structural packages and align with program manager Stantec and engineers AECOM/Jacobs.</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Metro Vancouver restructured the $6B project in late 2025 to rehabilitate the existing primary plant and deliver phased secondary-treatment upgrades; Phase 1 early-enabling works are wrapping up in 2026, with the bulk of heavy civil construction packages (treatment processes, new structures, marine infrastructure) expected to tender through 2026–2027 for a project running to 2035.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Baptiste Nickel Project – Mine Site Civil Infrastructure (FPX Nickel Corp., Fort St. James)</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>BC Government Major Projects / IAAC / EAO EPIC</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>https://www2.gov.bc.ca/gov/content/employment-business/major-projects</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Contact FPX Nickel Corp. directly in Vancouver to register as a civil/earthworks contractor of interest; review IAAC project file #90051 for scope detail and engage the Tl'azt'en Nation to understand Indigenous procurement requirements before formal RFQs are issued.</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>FPX Nickel's open-pit nickel mine 80 km northwest of Fort St. James received its final investment decision in September 2026 and is now under construction; BC's major-projects page confirms construction has commenced, requiring roads, earthworks, tailings facility, process plant, and a transmission line to a BC Hydro substation near Fraser Lake — a multi-year civil construction opportunity estimated at approximately $2.3B total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>RFQ 26-212 – Design and Construction Services, Brett Sewer Lift Station &amp; Force Main Upgrades (District of Saanich)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>MERX</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>https://www.merx.com/public/solicitations/british-columbia-379</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Download documents from MERX (solicitation 444184257075) and submit qualifications before October 29, 2026; coordinate with a registered BC civil engineering sub-consultant if design services are not in-house.</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>MERX-posted RFQ for design and construction of sewer lift station and force main upgrades in Saanich, BC — a civil/structural underground utilities opportunity closing October 29, 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Installation of Fuel Heaters, Burner Building, and Auxiliary Systems at Fort Nelson Gas (BC Hydro)</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>MERX / BC Hydro</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>https://www.merx.com/public/solicitations/british-columbia-379</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Register on BC Bid and access tender documents (MERX solicitation 444184257056); ensure COR certification and BC Hydro vendor pre-qualification are current before submitting. Contact BC Hydro Procurement for site clarification questions.</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>BC Hydro published an open tender on MERX on October 5, 2026 for mechanical/civil installation of fuel heaters, a burner building, and auxiliary systems at its Fort Nelson Gas facility — closing October 27, 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Regional Water Supply – Sooke Lake and Deception Watershed Dams: Seismic Assessment and Retrofit Design of Flow Control Infrastructure (Capital Regional District)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>MERX / Cornerstone Contracts</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>https://cornerstonecontracts.com/tenders/british-columbia</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Pull the full solicitation document from MERX immediately; assemble a team with dam-safety and seismic-retrofit credentials (P.Eng. BC-registered) and submit before October 14, 2026. Reference BC Dam Safety Regulation experience prominently.</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>CRD posted an open civil/structural engineering tender for seismic assessment and retrofit design of dam flow-control infrastructure — a specialist civil-structural engineering opportunity closing October 14, 2026 via MERX.</t>
         </is>
       </c>
     </row>
@@ -1665,7 +1917,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2204,13 +2456,11 @@
           <t>JDS Energy &amp; Mining — Project Delivery Leadership</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>JDS Energy &amp; Mining Inc.</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>GlobeNewswire / International Mining</t>
@@ -2221,8 +2471,6 @@
           <t>https://im-mining.com/2026/02/10/osisko-development-enlists-jds-for-cariboo-gold-project-build/</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -2250,13 +2498,11 @@
           <t>Leif Nilsson</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
           <t>Surge Copper Corp.</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>GlobeNewswire / Surge Copper</t>
@@ -2267,8 +2513,6 @@
           <t>https://www.globenewswire.com/news-release/2026/09/16/3363033/0/en/surge-copper-commences-environmental-assessment-process-for-berg-copper-project.html</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -2296,13 +2540,11 @@
           <t>Jeanine Martin</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
           <t>Vancouver Regional Construction Association (VRCA)</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>Journal of Commerce / VRCA</t>
@@ -2313,8 +2555,6 @@
           <t>https://canada.constructconnect.com/joc/news/government/2026/09/b-c-construction-leaders-seek-certainty-amid-election-instability</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -2328,6 +2568,144 @@
       <c r="L15" t="inlineStr">
         <is>
           <t>Jeanine Martin, as VRCA president, is leading the industry's post-election advocacy campaign for stable infrastructure procurement and prompt payment legislation in BC; she is actively meeting with all provincial party leaders and candidates ahead of the October 24, 2026 election and is a central connector to Metro Vancouver's major public client network, including TransLink, Metro Vancouver, and the BC Ministry of Transportation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Mark Liedemann</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Infrastructure BC</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Infrastructure BC / ReNew Canada</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>https://www.infrastructurebc.com/about/management-team/</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Contact Mark Liedemann via Infrastructure BC's Vancouver office (604-806-4168) or email Emily.Courville@infrastructurebc.com to request a briefing on upcoming Fraser River Tunnel GC-3 through GC-5 procurement timelines and to ensure your firm is on the project distribution list before RFQs are posted.</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Mark Liedemann leads BC's crown infrastructure procurement and delivery agency, which published the 2026 Spring BC Major Infrastructure Projects Brochure listing $52B in projects including the Fraser River Tunnel, Surrey-Langley SkyTrain, and Iona Island WWTP. Infrastructure BC is directly managing procurement for the re-tendered Fraser River Tunnel packages and sits at the nexus of every major P3/DB/DBF project in the province.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Jagrup Brar</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>BC Ministry of Mining and Critical Minerals</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>BC Gov News</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>https://news.gov.bc.ca/ministries/mining-and-critical-minerals/biography</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Write to MCM.Minister@gov.bc.ca (or call 250-953-0900) to request a meeting with ministry staff responsible for the Critical Minerals Office to understand the procurement calendar for newly permitted mine projects — particularly Baptiste Nickel, Mt. Milligan expansion, and Eskay Creek — and to register your firm as an interested civil contractor.</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Minister Brar's ministry directly controls exploration permitting timelines, the Critical Minerals Office (which is fast-tracking Baptiste Nickel and other projects), and is overseeing 17 projects advancing toward construction across northern BC. His ministry is the gateway for civil contractors seeking early positioning on mine-access road, tailings, and process facility packages for projects approved under the new fixed-timeline framework.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Todd Stone</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Association for Mineral Exploration (AME BC)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>AME BC / Business in Vancouver</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>https://amebc.ca/about/board-staff/</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Email Todd Stone at tstone@amebc.ca to introduce your firm's mine-site civil and infrastructure capabilities and request to be included in AME BC's contractor/supplier network communications; ask about presenting at an upcoming AME member event (e.g., the AME Roundup) to build visibility with exploration-company decision-makers ahead of upcoming construction procurement.</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Todd Stone, a former BC Minister of Transportation, took over as AME BC's president and CEO in August 2025 and represents more than 6,000 members engaged in mineral exploration and development across BC. AME BC is the fastest route to intelligence on which exploration-stage projects are moving toward pre-feasibility and construction, and Stone's government relationships make him a high-value connector to both ministry permitting staff and mining company proponents planning civil scopes.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update leads tracker 2026-10-14
</commit_message>
<xml_diff>
--- a/leads_tracker.xlsx
+++ b/leads_tracker.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M33"/>
+  <dimension ref="A1:M39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1640,11 +1640,6 @@
           <t>Fraser River Tunnel Project – Remaining Three Civil Construction Packages (GC-3 through GC-5)</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
           <t>BC Gov News / Infrastructure BC / ENR</t>
@@ -1687,11 +1682,6 @@
           <t>Iona Island Wastewater Treatment Plant Upgrade – Phase 2 Major Construction Packages (Metro Vancouver)</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
           <t>Metro Vancouver / Water Canada / ReNew Canada</t>
@@ -1734,11 +1724,6 @@
           <t>Baptiste Nickel Project – Mine Site Civil Infrastructure (FPX Nickel Corp., Fort St. James)</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
           <t>BC Government Major Projects / IAAC / EAO EPIC</t>
@@ -1781,11 +1766,6 @@
           <t>RFQ 26-212 – Design and Construction Services, Brett Sewer Lift Station &amp; Force Main Upgrades (District of Saanich)</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
           <t>MERX</t>
@@ -1828,11 +1808,6 @@
           <t>Installation of Fuel Heaters, Burner Building, and Auxiliary Systems at Fort Nelson Gas (BC Hydro)</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
           <t>MERX / BC Hydro</t>
@@ -1875,11 +1850,6 @@
           <t>Regional Water Supply – Sooke Lake and Deception Watershed Dams: Seismic Assessment and Retrofit Design of Flow Control Infrastructure (Capital Regional District)</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
           <t>MERX / Cornerstone Contracts</t>
@@ -1903,6 +1873,288 @@
       <c r="M33" t="inlineStr">
         <is>
           <t>CRD posted an open civil/structural engineering tender for seismic assessment and retrofit design of dam flow-control infrastructure — a specialist civil-structural engineering opportunity closing October 14, 2026 via MERX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Iona Island Wastewater Treatment Plant (IIWWTP) – Phase 2 Construction Packages (2027–2035)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Metro Vancouver Liquid Waste Committee / ReNew Canada</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>https://www.renewcanada.net/the-projects/iona-island-wastewater-treatment-plant/</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Register on Metro Vancouver's Bids &amp; Tenders portal and attend the next Liquid Waste Committee meeting (November update cycle) to track Stage Gate 2 (Detailed Design approval) — position now as a civil/structural sub or prime before shortlisting begins.</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Metro Vancouver's $6-billion upgrade of the Iona Island WWTP is now in preliminary design (10% complete); major civil, structural, mechanical, and process construction packages are expected to tender through 2027–2034, with specialized trades (electrical, mechanical, tunnelling) already flagged as labour-constrained.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>BC Hydro West End &amp; East Vancouver Underground Substation Projects (~$2.4B combined)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>BC Hydro / Journal of Commerce</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>https://canada.constructconnect.com/joc/news/infrastructure/2026/09/new-substations-slated-for-downtown-vancouver-one-will-be-built-underground</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Monitor the BCUC proceeding (Application in Progress) for the certificate decision expected by Oct 30, 2026; pre-qualify with BC Hydro's procurement team for civil underground and electrical infrastructure work — WSP holds the A&amp;E contract so approach them as a construction partner.</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>BC Hydro is awaiting a BCUC decision by October 30, 2026, to commence construction of two new Vancouver substations (West End ~$1B underground, East Vancouver ~$1B) with construction targeted to begin no earlier than late 2026 — civil/structural, deep excavation, and electrical packages will follow BCUC approval.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Berg Copper Project – Mine Site Civil &amp; Infrastructure Construction (EA Early Engagement Phase)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>EAO / Mining.com / IAAC Project Registry</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>https://iaac-aeic.gc.ca/050/evaluations/proj/90756</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Submit comments to EAO/IAAC before the November 9, 2026, deadline to establish your firm's presence early; reach out to Surge Copper's project team in Vancouver to discuss future engineering and civil construction scopes while the EA process advances.</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Surge Copper Corp. filed its Initial Project Description for the Berg open-pit copper-molybdenum mine (~80 km SW of Houston, BC) with the EAO and IAAC on September 9, 2026; the project includes a new 125-km transmission line to BC Hydro's grid, mine access roads, processing plant, and camp — early civil infrastructure tenders are 2–4 years out pending EA completion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>26-0244 – Engineering and Construction Services, Production Way Operations Center Renovation (Metro Vancouver)</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Metro Vancouver / Bids &amp; Tenders</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>https://metrovancouver.bidsandtenders.ca</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Download documents immediately from Metro Vancouver's Bids &amp; Tenders portal (Tender 26-0244); identify sub-trade partners for mechanical and electrical scope; attend any mandatory site meeting and submit before the December 18, 2026, closing date.</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Metro Vancouver has posted an open RFP for engineering and construction services for the renovation of its Production Way Operations Center — an active civil/structural and building renovation package closing December 18, 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>PS20261908-ENG-RFP – Consultant for Granville Bridge South Ramps Rehabilitation Phase 2 (City of Vancouver / MERX)</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>MERX / City of Vancouver</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>https://www.merx.com/public/solicitations/british-columbia-379</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Purchase documents on MERX immediately; assemble a structural engineering team with bridge rehabilitation experience; submit by October 20, 2026 — winning this positions your firm for the subsequent construction-phase contract.</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>The City of Vancouver has issued an RFP via MERX for a structural/civil engineering consultant to lead the Phase 2 rehabilitation of the Granville Bridge South Ramps — closing October 20, 2026, this is an immediate civil/structural engineering pursuit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>APN-AEC11 – Source Control (Design-Bid-Build), 19 Wing CFB Comox, Lazo, BC (Defence Construction Canada / MERX)</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>MERX / Defence Construction Canada</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>https://www.merx.com/dcc</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Register on the DCC electronic bidding site (merx.com/dcc) and download the APN documents; engage a geotechnical or environmental sub-consultant familiar with DND remediation work; submit before November 23, 2026.</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>Defence Construction Canada has issued an Advanced Procurement Notice for a design-bid-build heavy civil source-control project at CFB Comox on Vancouver Island, published October 9, 2026, closing November 23, 2026 — a federal heavy civil ground remediation opportunity.</t>
         </is>
       </c>
     </row>
@@ -1917,7 +2169,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2582,13 +2834,11 @@
           <t>Mark Liedemann</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
           <t>Infrastructure BC</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>Infrastructure BC / ReNew Canada</t>
@@ -2599,8 +2849,6 @@
           <t>https://www.infrastructurebc.com/about/management-team/</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -2628,13 +2876,11 @@
           <t>Jagrup Brar</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
           <t>BC Ministry of Mining and Critical Minerals</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>BC Gov News</t>
@@ -2645,8 +2891,6 @@
           <t>https://news.gov.bc.ca/ministries/mining-and-critical-minerals/biography</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -2674,13 +2918,11 @@
           <t>Todd Stone</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
           <t>Association for Mineral Exploration (AME BC)</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>AME BC / Business in Vancouver</t>
@@ -2691,8 +2933,6 @@
           <t>https://amebc.ca/about/board-staff/</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -2706,6 +2946,144 @@
       <c r="L18" t="inlineStr">
         <is>
           <t>Todd Stone, a former BC Minister of Transportation, took over as AME BC's president and CEO in August 2025 and represents more than 6,000 members engaged in mineral exploration and development across BC. AME BC is the fastest route to intelligence on which exploration-stage projects are moving toward pre-feasibility and construction, and Stone's government relationships make him a high-value connector to both ministry permitting staff and mining company proponents planning civil scopes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Andrew Osterloh</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Skeena Resources Ltd. (Gold &amp; Silver)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Skeena Resources / Northern Miner</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://secure.northernminer.com/news/</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Reach out via LinkedIn or Skeena's Vancouver corporate office this week — lead with your firm's remote site construction and commissioning experience in NW BC; reference Eskay's Q2 2027 first-ore target as the hook for urgency.</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Osterloh leads all engineering and construction activities at Skeena's Eskay Creek project, which is 70–75% complete with commissioning targeted for early 2027; remaining civil, electrical, and site infrastructure scopes are still being assigned to contractors and specialist suppliers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Gordon Doerksen</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Cambria Gold Mines Inc. (TSXV: CAMB)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Mining News North / BNN Bloomberg</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>https://www.bnnbloomberg.ca/press-releases/2026/10/05/cambria-gold-mines-announces-development-and-construction-update-at-red-mountain-and-premier-gold-projects-additions-to-engineering-team-and-warrants-exercised-to-date/</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Contact Doerksen at Cambria's Vancouver office this week — lead with heavy civil road construction capability in challenging mountain terrain; the haul-road permit application is being advanced now, making this the optimal window to pre-position as a preferred contractor.</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Doerksen is overseeing construction of the 23-km Red Mountain access road near Stewart, BC (Phase 1, 12 km to be completed by end of 2026, Phase 2 alpine road in 2027); a feasibility study update for four deposits is due Q4 2026, which will trigger haul-road permitting and broader mine-site civil construction packages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Leif Nilsson</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Surge Copper Corp. (TSXV: SURG)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>EAO / Globe Newswire / Surge Copper Corp.</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>https://www.globenewswire.com/news-release/2026/09/16/3363033/0/en/surge-copper-commences-environmental-assessment-process-for-berg-copper-project.html</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Submit a comment to the EAO/IAAC process before November 9 to establish visibility, then contact Surge's Vancouver head office to pitch environmental baseline, geotechnical, and early civil engineering services — the EA planning phase is actively underway and consultants are being engaged now.</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Surge's CEO is steering the Berg Copper Project (central BC open-pit Cu-Mo mine, pre-feasibility complete June 2026) through its formal EA process with EAO and IAAC, with public comment open until November 9, 2026 — the company needs environmental, civil engineering, and First Nations engagement consultants immediately for baseline studies and feasibility-level technical work.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update leads tracker 2026-10-21
</commit_message>
<xml_diff>
--- a/leads_tracker.xlsx
+++ b/leads_tracker.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M39"/>
+  <dimension ref="A1:M45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1892,11 +1892,6 @@
           <t>Iona Island Wastewater Treatment Plant (IIWWTP) – Phase 2 Construction Packages (2027–2035)</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
           <t>Metro Vancouver Liquid Waste Committee / ReNew Canada</t>
@@ -1939,11 +1934,6 @@
           <t>BC Hydro West End &amp; East Vancouver Underground Substation Projects (~$2.4B combined)</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
           <t>BC Hydro / Journal of Commerce</t>
@@ -1986,11 +1976,6 @@
           <t>Berg Copper Project – Mine Site Civil &amp; Infrastructure Construction (EA Early Engagement Phase)</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
           <t>EAO / Mining.com / IAAC Project Registry</t>
@@ -2033,11 +2018,6 @@
           <t>26-0244 – Engineering and Construction Services, Production Way Operations Center Renovation (Metro Vancouver)</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
           <t>Metro Vancouver / Bids &amp; Tenders</t>
@@ -2080,11 +2060,6 @@
           <t>PS20261908-ENG-RFP – Consultant for Granville Bridge South Ramps Rehabilitation Phase 2 (City of Vancouver / MERX)</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
           <t>MERX / City of Vancouver</t>
@@ -2127,11 +2102,6 @@
           <t>APN-AEC11 – Source Control (Design-Bid-Build), 19 Wing CFB Comox, Lazo, BC (Defence Construction Canada / MERX)</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
           <t>MERX / Defence Construction Canada</t>
@@ -2155,6 +2125,288 @@
       <c r="M39" t="inlineStr">
         <is>
           <t>Defence Construction Canada has issued an Advanced Procurement Notice for a design-bid-build heavy civil source-control project at CFB Comox on Vancouver Island, published October 9, 2026, closing November 23, 2026 — a federal heavy civil ground remediation opportunity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Fraser River Tunnel Project – Multiple Re-Tendered Civil Packages</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>ReNew Canada / BC Gov News</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>https://www.renewcanada.net/b-c-to-retender-contract-to-build-fraser-river-tunnel-project/</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Register on highway99tunnel.ca, monitor BC Bid for RFQ postings on tunnelling, marine, civil earthworks, and utility packages; position as a local BC contractor to leverage the province's explicit goal of increasing local participation.</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>BC MoTI cancelled its single design-build agreement with Cross Fraser Partnership and is re-tendering the $4.15B+ immersed-tube George Massey Tunnel replacement as multiple separate procurement packages; RFQs for key phases are expected imminently.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Berg Copper Project (Surge Copper Corp.) – $4.7B Mine Construction Pipeline</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>EAO Project Registry / Surge Copper Corp.</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>https://projects.eao.gov.bc.ca/</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Contact Surge Copper's EA representative Jennifer Anthony now to register as an interested contractor/consultant; target pre-qualification for access road, site prep, camp, tailings, and concentrator civil packages ahead of a potential 2028–2029 construction award.</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Surge Copper's 100%-owned Berg open-pit copper-molybdenum mine near Houston, BC entered EAO/IAAC public comment on Oct. 8, 2026; the PFS defines a 3-year, C$4.7B initial capital build with a 28-year mine life, and Surge is now advancing feasibility-level engineering and environmental baseline studies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>FortisBC Tilbury Phase 2 LNG Expansion – $3B–$6B Heavy Civil &amp; Industrial</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Journal of Commerce (ConstructConnect) / BC Gov News</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>https://canada.constructconnect.com/joc/news/infrastructure/2026/09/province-issues-ea-certificate-for-tilbury-phase-2-lng-expansion</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Contact FortisBC's major projects procurement team directly; no general contracts have been awarded yet. Position now for civil earthworks, marine jetty, mechanical, and tankage packages before the 2027 FEED-to-EPC transition.</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>FortisBC received its provincial EA certificate and federal approval in September 2026 for the Tilbury Island Phase 2 expansion in Delta; facility construction could start as early as mid-2027, generating ~6,200 FTE years of employment including new LNG storage tank, liquefaction train, and a marine jetty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Consulting Engineering Services – Detailed Design, Construction &amp; Decommissioning of Sapperton Pump Station (Metro Vancouver RFP 26-0444)</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>MERX / Metro Vancouver Bids &amp; Tenders</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>https://www.merx.com/public/solicitations/british-columbia-379</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Download documents immediately from metrovancouver.org/bidding-opportunities; assemble a team with liquid-waste pump station experience (e.g., mechanical-process, geotechnical, electrical) — AECOM, Brown and Caldwell, and Stantec are known incumbents so differentiate on local staffing and First Nations engagement.</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>Metro Vancouver is seeking a civil/structural engineering consultant to lead detailed design, construction administration, and decommissioning of the Sapperton Pump Station in New Westminster; published Oct. 19, 2026, closing Nov. 19, 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>APN – Construction Management Services, Mainland BC Infrastructure Modernization (Defence Construction Canada – Pacific Region)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>MERX</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>https://www.merx.com/public/solicitations/british-columbia-379</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Register on MERX and download the APN (ref 4135752620); submit a Statement of Qualifications highlighting federal ICI experience, COR certification, and security clearance capacity to maximize shortlist standing before the formal RFP is released.</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>Defence Construction Canada Pacific Region posted an Advance Procurement Notice for Construction Management Services covering mainland BC federal infrastructure modernization; published Oct. 16, 2026, closing Nov. 25, 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Civil Engineering Consulting Services – Mountain Highway Improvements, Arborlynn Dr to Hwy 1 WB Ramps (District of North Vancouver RFP-066-26)</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>MERX / TenderScan</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>https://tenderscan.ca/tenders/vancouver/engineering-architecture</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Download RFP-066-26 from the District of North Vancouver portal; pair a transportation engineer with traffic modeling and MoTI interchange experience — highlight any prior North Shore or Highway 1 interchange work in your technical proposal.</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>District of North Vancouver is seeking a civil engineering consultant for road design and improvements on Mountain Highway between Arborlynn Drive and the Highway 1 westbound ramps; closing Nov. 6, 2026.</t>
         </is>
       </c>
     </row>
@@ -2169,7 +2421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2960,13 +3212,11 @@
           <t>Andrew Osterloh</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
           <t>Skeena Resources Ltd. (Gold &amp; Silver)</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>Skeena Resources / Northern Miner</t>
@@ -2977,8 +3227,6 @@
           <t>https://secure.northernminer.com/news/</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -3006,13 +3254,11 @@
           <t>Gordon Doerksen</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
           <t>Cambria Gold Mines Inc. (TSXV: CAMB)</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>Mining News North / BNN Bloomberg</t>
@@ -3023,8 +3269,6 @@
           <t>https://www.bnnbloomberg.ca/press-releases/2026/10/05/cambria-gold-mines-announces-development-and-construction-update-at-red-mountain-and-premier-gold-projects-additions-to-engineering-team-and-warrants-exercised-to-date/</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -3052,13 +3296,11 @@
           <t>Leif Nilsson</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
           <t>Surge Copper Corp. (TSXV: SURG)</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>EAO / Globe Newswire / Surge Copper Corp.</t>
@@ -3069,8 +3311,6 @@
           <t>https://www.globenewswire.com/news-release/2026/09/16/3363033/0/en/surge-copper-commences-environmental-assessment-process-for-berg-copper-project.html</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -3084,6 +3324,144 @@
       <c r="L21" t="inlineStr">
         <is>
           <t>Surge's CEO is steering the Berg Copper Project (central BC open-pit Cu-Mo mine, pre-feasibility complete June 2026) through its formal EA process with EAO and IAAC, with public comment open until November 9, 2026 — the company needs environmental, civil engineering, and First Nations engagement consultants immediately for baseline studies and feasibility-level technical work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Albert Au</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>BC Hydro</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Read Site News – People Moves August 2026</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://readsitenews.com/people-moves-august-2026/</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Send a congratulatory LinkedIn message referencing BC Hydro's active civil capital construction services standing offer (last issued July 2026 on CanadaBuys) and request a 20-minute intro call to discuss your firm's capabilities for upcoming dam safety, substation civil, and transmission line work.</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Albert Au was recently promoted to Manager, Supply Chain Infrastructure Projects at BC Hydro, making him the key gatekeeper for civil capital construction vendor selection and standing offer renewals at one of BC's largest infrastructure owners.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Greg Northcott</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Allnorth Consultants</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Read Site News – People Moves August 2026</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>https://readsitenews.com/people-moves-august-2026/</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Reach out via LinkedIn with a brief note on shared BC mining/civil markets (Berg, Schaft Creek, Red Chris) and request a meeting to explore teaming arrangements on upcoming EPC and EPCM bids where Allnorth's engineering depth complements heavy civil construction capacity.</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Greg Northcott was appointed CEO of Allnorth Consultants (a multi-discipline engineering and project services firm active in BC mining, energy, and heavy civil) effective August 17, 2026, bringing 25+ years of experience across engineering, construction, and environmental services in Canada — a new CEO typically initiates partnership and teaming conversations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Prab Sekhon, P.Eng.</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Seko Construction</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Read Site News – People Moves August 2026</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>https://readsitenews.com/people-moves-august-2026/</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Connect with Prab on LinkedIn, congratulate him on the promotion, and propose a meeting to discuss sub-trade or joint-venture opportunities on Metro Vancouver liquid waste, BC MoTI, or municipal heavy civil tenders where Seko is likely bidding as GC.</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Prab Sekhon was recently promoted from Project Manager to Director of Construction at Seko Construction's Vancouver office; Seko is an active BC general and civil contractor — a newly elevated Director of Construction typically seeks new sub-trade and teaming partners to build out their project delivery bench.</t>
         </is>
       </c>
     </row>

</xml_diff>